<commit_message>
MIX-KATA v2: Bobo, KURANG TEPAT + cuba lagi, lagu, latar kedai, genggam tangan, L3 dua jawapan
- Salah suap tidak lagi kalah: papar KURANG TEPAT, cawan melantun balik, nyawa -6
- Intro Bobo bercakap (3 ayat, taip + bunyi suara), latar kedai dengan kaunter
- Lagu latar ceria (Web Audio) makin laju ikut level, butang lagu/bunyi
- Kawalan tangan: genggam untuk pegang, buka untuk lepas (bukan cubit)
- Level 3: 4 pilihan, 2 jawapan betul; templat terima jawapan 'A,C'

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P981k1QsTFpp6CPgxFuC7n
</commit_message>
<xml_diff>
--- a/public/templates/templat-mixkata.xlsx
+++ b/public/templates/templat-mixkata.xlsx
@@ -405,7 +405,7 @@
     <col min="4" max="4" width="16.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,7 +428,7 @@
         <v>Pilihan D</v>
       </c>
       <c r="G1" t="str">
-        <v>Jawapan Betul (A/B/C/D)</v>
+        <v>Jawapan Betul (cth: A atau A,C)</v>
       </c>
     </row>
     <row r="2">
@@ -436,7 +436,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Si Bubu mahu minuman KATA GANDA! Suap cawan yang betul.</v>
+        <v>Bobo haus! Suapkan air KATA GANDA.</v>
       </c>
       <c r="C2" t="str">
         <v>roti-roti</v>
@@ -459,7 +459,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>Cawan manakah KATA GANDA?</v>
+        <v>Air manakah KATA GANDA?</v>
       </c>
       <c r="C3" t="str">
         <v>kedai</v>
@@ -482,7 +482,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="str">
-        <v>Cawan manakah KATA GANDA?</v>
+        <v>Air manakah KATA GANDA?</v>
       </c>
       <c r="C4" t="str">
         <v>cawan</v>
@@ -505,7 +505,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="str">
-        <v>Si Bubu lapar! Suap cawan KATA GANDA.</v>
+        <v>Tolong Bobo! Suapkan air KATA GANDA.</v>
       </c>
       <c r="C5" t="str">
         <v>pagi-pagi</v>
@@ -528,22 +528,22 @@
         <v>3</v>
       </c>
       <c r="B6" t="str">
-        <v>Cawan manakah KATA GANDA?</v>
+        <v>Ada DUA air KATA GANDA! Suapkan kedua-duanya.</v>
       </c>
       <c r="C6" t="str">
-        <v>duit</v>
+        <v>duit-duit</v>
       </c>
       <c r="D6" t="str">
         <v>baki</v>
       </c>
       <c r="E6" t="str">
-        <v>duit-duit</v>
+        <v>kuih-kuih</v>
       </c>
       <c r="F6" t="str">
         <v>pembeli</v>
       </c>
       <c r="G6" t="str">
-        <v>C</v>
+        <v>A,C</v>
       </c>
     </row>
     <row r="7">
@@ -551,22 +551,22 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>Cepat! Suap cawan KATA GANDA.</v>
+        <v>Cari DUA air KATA GANDA untuk Bobo.</v>
       </c>
       <c r="C7" t="str">
-        <v>kuih-kuih</v>
+        <v>kedai</v>
       </c>
       <c r="D7" t="str">
-        <v>kuih</v>
+        <v>gelas-gelas</v>
       </c>
       <c r="E7" t="str">
-        <v>kek</v>
+        <v>minuman</v>
       </c>
       <c r="F7" t="str">
-        <v>kedai</v>
+        <v>botol-botol</v>
       </c>
       <c r="G7" t="str">
-        <v>A</v>
+        <v>B,D</v>
       </c>
     </row>
     <row r="8">
@@ -574,7 +574,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="str">
-        <v>Hati-hati! Yang mana kata ganda yang BETUL?</v>
+        <v>Hati-hati! Pilih DUA kata ganda yang BETUL.</v>
       </c>
       <c r="C8" t="str">
         <v>kawan kawan</v>
@@ -583,13 +583,13 @@
         <v>kawan-kawan</v>
       </c>
       <c r="E8" t="str">
+        <v>cawan-cawan</v>
+      </c>
+      <c r="F8" t="str">
         <v>berkawan</v>
       </c>
-      <c r="F8" t="str">
-        <v>kawan</v>
-      </c>
       <c r="G8" t="str">
-        <v>B</v>
+        <v>B,C</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIX-KATA v2: Bobo, KURANG TEPAT + cuba lagi, lagu, latar kedai, genggam tangan, L3 dua jawapan (#2)
- Salah suap tidak lagi kalah: papar KURANG TEPAT, cawan melantun balik, nyawa -6
- Intro Bobo bercakap (3 ayat, taip + bunyi suara), latar kedai dengan kaunter
- Lagu latar ceria (Web Audio) makin laju ikut level, butang lagu/bunyi
- Kawalan tangan: genggam untuk pegang, buka untuk lepas (bukan cubit)
- Level 3: 4 pilihan, 2 jawapan betul; templat terima jawapan 'A,C'


Claude-Session: https://claude.ai/code/session_01P981k1QsTFpp6CPgxFuC7n

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/templat-mixkata.xlsx
+++ b/public/templates/templat-mixkata.xlsx
@@ -405,7 +405,7 @@
     <col min="4" max="4" width="16.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,7 +428,7 @@
         <v>Pilihan D</v>
       </c>
       <c r="G1" t="str">
-        <v>Jawapan Betul (A/B/C/D)</v>
+        <v>Jawapan Betul (cth: A atau A,C)</v>
       </c>
     </row>
     <row r="2">
@@ -436,7 +436,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Si Bubu mahu minuman KATA GANDA! Suap cawan yang betul.</v>
+        <v>Bobo haus! Suapkan air KATA GANDA.</v>
       </c>
       <c r="C2" t="str">
         <v>roti-roti</v>
@@ -459,7 +459,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>Cawan manakah KATA GANDA?</v>
+        <v>Air manakah KATA GANDA?</v>
       </c>
       <c r="C3" t="str">
         <v>kedai</v>
@@ -482,7 +482,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="str">
-        <v>Cawan manakah KATA GANDA?</v>
+        <v>Air manakah KATA GANDA?</v>
       </c>
       <c r="C4" t="str">
         <v>cawan</v>
@@ -505,7 +505,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="str">
-        <v>Si Bubu lapar! Suap cawan KATA GANDA.</v>
+        <v>Tolong Bobo! Suapkan air KATA GANDA.</v>
       </c>
       <c r="C5" t="str">
         <v>pagi-pagi</v>
@@ -528,22 +528,22 @@
         <v>3</v>
       </c>
       <c r="B6" t="str">
-        <v>Cawan manakah KATA GANDA?</v>
+        <v>Ada DUA air KATA GANDA! Suapkan kedua-duanya.</v>
       </c>
       <c r="C6" t="str">
-        <v>duit</v>
+        <v>duit-duit</v>
       </c>
       <c r="D6" t="str">
         <v>baki</v>
       </c>
       <c r="E6" t="str">
-        <v>duit-duit</v>
+        <v>kuih-kuih</v>
       </c>
       <c r="F6" t="str">
         <v>pembeli</v>
       </c>
       <c r="G6" t="str">
-        <v>C</v>
+        <v>A,C</v>
       </c>
     </row>
     <row r="7">
@@ -551,22 +551,22 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>Cepat! Suap cawan KATA GANDA.</v>
+        <v>Cari DUA air KATA GANDA untuk Bobo.</v>
       </c>
       <c r="C7" t="str">
-        <v>kuih-kuih</v>
+        <v>kedai</v>
       </c>
       <c r="D7" t="str">
-        <v>kuih</v>
+        <v>gelas-gelas</v>
       </c>
       <c r="E7" t="str">
-        <v>kek</v>
+        <v>minuman</v>
       </c>
       <c r="F7" t="str">
-        <v>kedai</v>
+        <v>botol-botol</v>
       </c>
       <c r="G7" t="str">
-        <v>A</v>
+        <v>B,D</v>
       </c>
     </row>
     <row r="8">
@@ -574,7 +574,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="str">
-        <v>Hati-hati! Yang mana kata ganda yang BETUL?</v>
+        <v>Hati-hati! Pilih DUA kata ganda yang BETUL.</v>
       </c>
       <c r="C8" t="str">
         <v>kawan kawan</v>
@@ -583,13 +583,13 @@
         <v>kawan-kawan</v>
       </c>
       <c r="E8" t="str">
+        <v>cawan-cawan</v>
+      </c>
+      <c r="F8" t="str">
         <v>berkawan</v>
       </c>
-      <c r="F8" t="str">
-        <v>kawan</v>
-      </c>
       <c r="G8" t="str">
-        <v>B</v>
+        <v>B,C</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Kaunter Lapar ringkas: tanpa soalan/pusingan/pemenang, MULA 3-2-1, pemasa jam sebenar; MIX-KATA buang pembayang 2 jawapan
- Kaunter Lapar: buang banner soalan, label pusingan, senarai pemenang & kedudukan;
  tamat masa hanya tunjuk watak (kenyang/pengsan) + butang MULA LAGI;
  kiraan 3-2-1 besar kekal di skrin; pemasa ikut jam sebenar
- MIX-KATA: buang label 'Ada 2 jawapan betul / tinggal', teks level & soalan
  asal tidak lagi sebut bilangan jawapan

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P981k1QsTFpp6CPgxFuC7n
</commit_message>
<xml_diff>
--- a/public/templates/templat-mixkata.xlsx
+++ b/public/templates/templat-mixkata.xlsx
@@ -528,7 +528,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="str">
-        <v>Ada DUA air KATA GANDA! Suapkan kedua-duanya.</v>
+        <v>Suapkan air KATA GANDA kepada Bobo.</v>
       </c>
       <c r="C6" t="str">
         <v>duit-duit</v>
@@ -551,7 +551,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>Cari DUA air KATA GANDA untuk Bobo.</v>
+        <v>Cari air KATA GANDA untuk Bobo.</v>
       </c>
       <c r="C7" t="str">
         <v>kedai</v>
@@ -574,7 +574,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="str">
-        <v>Hati-hati! Pilih DUA kata ganda yang BETUL.</v>
+        <v>Hati-hati! Pilih kata ganda yang BETUL.</v>
       </c>
       <c r="C8" t="str">
         <v>kawan kawan</v>

</xml_diff>

<commit_message>
Kaunter Lapar ringkas: tanpa soalan/pusingan/pemenang, MULA 3-2-1, pemasa jam sebenar; MIX-KATA buang pembayang 2 jawapan (#4)
- Kaunter Lapar: buang banner soalan, label pusingan, senarai pemenang & kedudukan;
  tamat masa hanya tunjuk watak (kenyang/pengsan) + butang MULA LAGI;
  kiraan 3-2-1 besar kekal di skrin; pemasa ikut jam sebenar
- MIX-KATA: buang label 'Ada 2 jawapan betul / tinggal', teks level & soalan
  asal tidak lagi sebut bilangan jawapan


Claude-Session: https://claude.ai/code/session_01P981k1QsTFpp6CPgxFuC7n

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/templat-mixkata.xlsx
+++ b/public/templates/templat-mixkata.xlsx
@@ -528,7 +528,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="str">
-        <v>Ada DUA air KATA GANDA! Suapkan kedua-duanya.</v>
+        <v>Suapkan air KATA GANDA kepada Bobo.</v>
       </c>
       <c r="C6" t="str">
         <v>duit-duit</v>
@@ -551,7 +551,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>Cari DUA air KATA GANDA untuk Bobo.</v>
+        <v>Cari air KATA GANDA untuk Bobo.</v>
       </c>
       <c r="C7" t="str">
         <v>kedai</v>
@@ -574,7 +574,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="str">
-        <v>Hati-hati! Pilih DUA kata ganda yang BETUL.</v>
+        <v>Hati-hati! Pilih kata ganda yang BETUL.</v>
       </c>
       <c r="C8" t="str">
         <v>kawan kawan</v>

</xml_diff>

<commit_message>
MIX-KATA: mod petikan ejaan (SP 3.3.2) + pilihan set soalan
- Soalan boleh ada petikan: dipaparkan besar pada papan 'Nota Bobo', Bobo
  beralih ke kanan; murid suap cawan perkataan SALAH EJAAN; bila betul,
  perkataan dalam petikan bertukar kepada ejaan betul (hijau)
- Set asal baharu: 7 petikan ejaan mudah Tahun 2 bertema Bobo/kedai/integriti
  (L1 2 cawan, L2 3 cawan, L3 4 cawan 2 salah); set Kata Ganda dikekalkan
- Menu: pilih set soalan (Ejaan / Kata Ganda / Soalan saya)
- Templat: lajur Petikan & Ejaan Betul (pilihan)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P981k1QsTFpp6CPgxFuC7n
</commit_message>
<xml_diff>
--- a/public/templates/templat-mixkata.xlsx
+++ b/public/templates/templat-mixkata.xlsx
@@ -397,15 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:I9"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="48.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -416,19 +418,25 @@
         <v>Soalan</v>
       </c>
       <c r="C1" t="str">
+        <v>Petikan (pilihan)</v>
+      </c>
+      <c r="D1" t="str">
         <v>Pilihan A</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Pilihan B</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Pilihan C</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Pilihan D</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Jawapan Betul (cth: A atau A,C)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Ejaan Betul (pilihan)</v>
       </c>
     </row>
     <row r="2">
@@ -436,22 +444,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Bobo haus! Suapkan air KATA GANDA.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C2" t="str">
-        <v>roti-roti</v>
+        <v>Bobo pergi ke kedai. Dia mahu membeli aiskrem.</v>
       </c>
       <c r="D2" t="str">
-        <v>roti</v>
+        <v>aiskrem</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>kedai</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
         <v>A</v>
+      </c>
+      <c r="I2" t="str">
+        <v>aiskrim</v>
       </c>
     </row>
     <row r="3">
@@ -459,22 +473,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>Air manakah KATA GANDA?</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C3" t="str">
-        <v>kedai</v>
+        <v>Bobo beratur dengan sabar di kaunter. Dia tidak memotong barisn.</v>
       </c>
       <c r="D3" t="str">
-        <v>kawan-kawan</v>
+        <v>kaunter</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>barisn</v>
       </c>
       <c r="F3" t="str">
         <v/>
       </c>
       <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
         <v>B</v>
+      </c>
+      <c r="I3" t="str">
+        <v>barisan</v>
       </c>
     </row>
     <row r="4">
@@ -482,22 +502,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="str">
-        <v>Air manakah KATA GANDA?</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C4" t="str">
-        <v>cawan</v>
+        <v>Bobo membeli segelas air teh. Harganya lima ringit. Dia membayar dengan duit kertas.</v>
       </c>
       <c r="D4" t="str">
-        <v>cawan-cawan</v>
+        <v>segelas</v>
       </c>
       <c r="E4" t="str">
-        <v>minuman</v>
+        <v>ringit</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>kertas</v>
       </c>
       <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
         <v>B</v>
+      </c>
+      <c r="I4" t="str">
+        <v>ringgit</v>
       </c>
     </row>
     <row r="5">
@@ -505,22 +531,28 @@
         <v>2</v>
       </c>
       <c r="B5" t="str">
-        <v>Tolong Bobo! Suapkan air KATA GANDA.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C5" t="str">
-        <v>pagi-pagi</v>
+        <v>Penjual memberikan baki kepada Bobo. Bobo mengucapkan terima kaseh.</v>
       </c>
       <c r="D5" t="str">
-        <v>pagi</v>
+        <v>baki</v>
       </c>
       <c r="E5" t="str">
-        <v>petang</v>
+        <v>penjual</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>kaseh</v>
       </c>
       <c r="G5" t="str">
-        <v>A</v>
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>C</v>
+      </c>
+      <c r="I5" t="str">
+        <v>kasih</v>
       </c>
     </row>
     <row r="6">
@@ -528,22 +560,28 @@
         <v>3</v>
       </c>
       <c r="B6" t="str">
-        <v>Suapkan air KATA GANDA kepada Bobo.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C6" t="str">
-        <v>duit-duit</v>
+        <v>Penjual tersalah memberi baki. Bobo memulangkan duit itu kerana dia jujor. Penjual itu sangat gembera.</v>
       </c>
       <c r="D6" t="str">
+        <v>jujor</v>
+      </c>
+      <c r="E6" t="str">
+        <v>penjual</v>
+      </c>
+      <c r="F6" t="str">
+        <v>gembera</v>
+      </c>
+      <c r="G6" t="str">
         <v>baki</v>
       </c>
-      <c r="E6" t="str">
-        <v>kuih-kuih</v>
-      </c>
-      <c r="F6" t="str">
-        <v>pembeli</v>
-      </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>A,C</v>
+      </c>
+      <c r="I6" t="str">
+        <v>jujur, gembira</v>
       </c>
     </row>
     <row r="7">
@@ -551,22 +589,28 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>Cari air KATA GANDA untuk Bobo.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C7" t="str">
-        <v>kedai</v>
+        <v>Bobo minum air teh yang sejok. Dia membuang cawan ke dalam tong sampa. Bobo budak yang bersih.</v>
       </c>
       <c r="D7" t="str">
-        <v>gelas-gelas</v>
+        <v>cawan</v>
       </c>
       <c r="E7" t="str">
-        <v>minuman</v>
+        <v>sejok</v>
       </c>
       <c r="F7" t="str">
-        <v>botol-botol</v>
+        <v>bersih</v>
       </c>
       <c r="G7" t="str">
+        <v>sampa</v>
+      </c>
+      <c r="H7" t="str">
         <v>B,D</v>
+      </c>
+      <c r="I7" t="str">
+        <v>sejuk, sampah</v>
       </c>
     </row>
     <row r="8">
@@ -574,27 +618,62 @@
         <v>3</v>
       </c>
       <c r="B8" t="str">
-        <v>Hati-hati! Pilih kata ganda yang BETUL.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C8" t="str">
-        <v>kawan kawan</v>
+        <v>Bobo membeli dua biji rotti dan sebotol air. Dia membawa beg plastik. Bobo berjalan pulang ke rumh.</v>
       </c>
       <c r="D8" t="str">
+        <v>rotti</v>
+      </c>
+      <c r="E8" t="str">
+        <v>plastik</v>
+      </c>
+      <c r="F8" t="str">
+        <v>berjalan</v>
+      </c>
+      <c r="G8" t="str">
+        <v>rumh</v>
+      </c>
+      <c r="H8" t="str">
+        <v>A,D</v>
+      </c>
+      <c r="I8" t="str">
+        <v>roti, rumah</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Contoh TANPA petikan (kata ganda): Air manakah KATA GANDA?</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>kedai</v>
+      </c>
+      <c r="E9" t="str">
         <v>kawan-kawan</v>
       </c>
-      <c r="E8" t="str">
-        <v>cawan-cawan</v>
-      </c>
-      <c r="F8" t="str">
-        <v>berkawan</v>
-      </c>
-      <c r="G8" t="str">
-        <v>B,C</v>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>B</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MIX-KATA: mod petikan ejaan (SP 3.3.2) + pilihan set soalan (#6)
- Soalan boleh ada petikan: dipaparkan besar pada papan 'Nota Bobo', Bobo
  beralih ke kanan; murid suap cawan perkataan SALAH EJAAN; bila betul,
  perkataan dalam petikan bertukar kepada ejaan betul (hijau)
- Set asal baharu: 7 petikan ejaan mudah Tahun 2 bertema Bobo/kedai/integriti
  (L1 2 cawan, L2 3 cawan, L3 4 cawan 2 salah); set Kata Ganda dikekalkan
- Menu: pilih set soalan (Ejaan / Kata Ganda / Soalan saya)
- Templat: lajur Petikan & Ejaan Betul (pilihan)


Claude-Session: https://claude.ai/code/session_01P981k1QsTFpp6CPgxFuC7n

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/templat-mixkata.xlsx
+++ b/public/templates/templat-mixkata.xlsx
@@ -397,15 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:I9"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="48.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -416,19 +418,25 @@
         <v>Soalan</v>
       </c>
       <c r="C1" t="str">
+        <v>Petikan (pilihan)</v>
+      </c>
+      <c r="D1" t="str">
         <v>Pilihan A</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Pilihan B</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Pilihan C</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Pilihan D</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Jawapan Betul (cth: A atau A,C)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Ejaan Betul (pilihan)</v>
       </c>
     </row>
     <row r="2">
@@ -436,22 +444,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Bobo haus! Suapkan air KATA GANDA.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C2" t="str">
-        <v>roti-roti</v>
+        <v>Bobo pergi ke kedai. Dia mahu membeli aiskrem.</v>
       </c>
       <c r="D2" t="str">
-        <v>roti</v>
+        <v>aiskrem</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>kedai</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
         <v>A</v>
+      </c>
+      <c r="I2" t="str">
+        <v>aiskrim</v>
       </c>
     </row>
     <row r="3">
@@ -459,22 +473,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>Air manakah KATA GANDA?</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C3" t="str">
-        <v>kedai</v>
+        <v>Bobo beratur dengan sabar di kaunter. Dia tidak memotong barisn.</v>
       </c>
       <c r="D3" t="str">
-        <v>kawan-kawan</v>
+        <v>kaunter</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>barisn</v>
       </c>
       <c r="F3" t="str">
         <v/>
       </c>
       <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
         <v>B</v>
+      </c>
+      <c r="I3" t="str">
+        <v>barisan</v>
       </c>
     </row>
     <row r="4">
@@ -482,22 +502,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="str">
-        <v>Air manakah KATA GANDA?</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C4" t="str">
-        <v>cawan</v>
+        <v>Bobo membeli segelas air teh. Harganya lima ringit. Dia membayar dengan duit kertas.</v>
       </c>
       <c r="D4" t="str">
-        <v>cawan-cawan</v>
+        <v>segelas</v>
       </c>
       <c r="E4" t="str">
-        <v>minuman</v>
+        <v>ringit</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>kertas</v>
       </c>
       <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
         <v>B</v>
+      </c>
+      <c r="I4" t="str">
+        <v>ringgit</v>
       </c>
     </row>
     <row r="5">
@@ -505,22 +531,28 @@
         <v>2</v>
       </c>
       <c r="B5" t="str">
-        <v>Tolong Bobo! Suapkan air KATA GANDA.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C5" t="str">
-        <v>pagi-pagi</v>
+        <v>Penjual memberikan baki kepada Bobo. Bobo mengucapkan terima kaseh.</v>
       </c>
       <c r="D5" t="str">
-        <v>pagi</v>
+        <v>baki</v>
       </c>
       <c r="E5" t="str">
-        <v>petang</v>
+        <v>penjual</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>kaseh</v>
       </c>
       <c r="G5" t="str">
-        <v>A</v>
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>C</v>
+      </c>
+      <c r="I5" t="str">
+        <v>kasih</v>
       </c>
     </row>
     <row r="6">
@@ -528,22 +560,28 @@
         <v>3</v>
       </c>
       <c r="B6" t="str">
-        <v>Suapkan air KATA GANDA kepada Bobo.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C6" t="str">
-        <v>duit-duit</v>
+        <v>Penjual tersalah memberi baki. Bobo memulangkan duit itu kerana dia jujor. Penjual itu sangat gembera.</v>
       </c>
       <c r="D6" t="str">
+        <v>jujor</v>
+      </c>
+      <c r="E6" t="str">
+        <v>penjual</v>
+      </c>
+      <c r="F6" t="str">
+        <v>gembera</v>
+      </c>
+      <c r="G6" t="str">
         <v>baki</v>
       </c>
-      <c r="E6" t="str">
-        <v>kuih-kuih</v>
-      </c>
-      <c r="F6" t="str">
-        <v>pembeli</v>
-      </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>A,C</v>
+      </c>
+      <c r="I6" t="str">
+        <v>jujur, gembira</v>
       </c>
     </row>
     <row r="7">
@@ -551,22 +589,28 @@
         <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>Cari air KATA GANDA untuk Bobo.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C7" t="str">
-        <v>kedai</v>
+        <v>Bobo minum air teh yang sejok. Dia membuang cawan ke dalam tong sampa. Bobo budak yang bersih.</v>
       </c>
       <c r="D7" t="str">
-        <v>gelas-gelas</v>
+        <v>cawan</v>
       </c>
       <c r="E7" t="str">
-        <v>minuman</v>
+        <v>sejok</v>
       </c>
       <c r="F7" t="str">
-        <v>botol-botol</v>
+        <v>bersih</v>
       </c>
       <c r="G7" t="str">
+        <v>sampa</v>
+      </c>
+      <c r="H7" t="str">
         <v>B,D</v>
+      </c>
+      <c r="I7" t="str">
+        <v>sejuk, sampah</v>
       </c>
     </row>
     <row r="8">
@@ -574,27 +618,62 @@
         <v>3</v>
       </c>
       <c r="B8" t="str">
-        <v>Hati-hati! Pilih kata ganda yang BETUL.</v>
+        <v>Cari perkataan yang SALAH EJAAN dalam petikan!</v>
       </c>
       <c r="C8" t="str">
-        <v>kawan kawan</v>
+        <v>Bobo membeli dua biji rotti dan sebotol air. Dia membawa beg plastik. Bobo berjalan pulang ke rumh.</v>
       </c>
       <c r="D8" t="str">
+        <v>rotti</v>
+      </c>
+      <c r="E8" t="str">
+        <v>plastik</v>
+      </c>
+      <c r="F8" t="str">
+        <v>berjalan</v>
+      </c>
+      <c r="G8" t="str">
+        <v>rumh</v>
+      </c>
+      <c r="H8" t="str">
+        <v>A,D</v>
+      </c>
+      <c r="I8" t="str">
+        <v>roti, rumah</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Contoh TANPA petikan (kata ganda): Air manakah KATA GANDA?</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>kedai</v>
+      </c>
+      <c r="E9" t="str">
         <v>kawan-kawan</v>
       </c>
-      <c r="E8" t="str">
-        <v>cawan-cawan</v>
-      </c>
-      <c r="F8" t="str">
-        <v>berkawan</v>
-      </c>
-      <c r="G8" t="str">
-        <v>B,C</v>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>B</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>